<commit_message>
fix: improve readability and spacing
improve readability and spacing, remove legacy formula in Raging Smash
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/skills.xlsx
+++ b/mod_project/data_tables/skills.xlsx
@@ -547,13 +547,13 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Attract single-target attacks to user with high speed turn recovery.</t>
+          <t>Attract single-target attacks to user. High turn speed recovery.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Turns: 3 (L1) -&gt; 4 (L2) -&gt; 5 (L3) -&gt; 6 (L4) -&gt; 7 (L5 Max).
-Speed: +50% -&gt; +63% -&gt; +76% -&gt; +89% -&gt; +100%. TP: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5.</t>
+          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-L5)    |    Speed: +50% -&gt; +100%
+TP Cost: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -651,13 +651,13 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Raise party physical ATK &amp; replace debuffs. Usable out of battle.</t>
+          <t>Raise party physical ATK &amp; cleanse debuffs. Usable out of battle.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ATK: +8% (L1) -&gt; +10% (L2) -&gt; +12% (L3) -&gt; +14% (L4) -&gt; +18% (L5 Max).
-Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8. TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13.</t>
+          <t>ATK: +8% -&gt; +10% -&gt; +12% -&gt; +14% -&gt; +18% (L1-L5 Max)
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8    |    TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -711,13 +711,13 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Short-range skill. Strike one enemy for 125% ATK (+8%/Lv, Max 200%).</t>
+          <t>Short-range strike. Boosted accuracy (+20% to +38%). Delay: 0.80x.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Hit Rate: +20% (+2%/Lv, Max +38%). Action delay: 0.80x~0.90x.
-TP Cost: 5 (Lv1) -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 (Max).</t>
+          <t>ATK: 125% (L1) -&gt; 133 -&gt; 141 -&gt; 150 -&gt; 158 -&gt; 166 -&gt; 175 -&gt; 183 -&gt; 191 -&gt; 200% (L10)
+TP Cost: 5 (L1) -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 (Max)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -864,8 +864,8 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>DEF: +20% (L1) -&gt; +27% (L2) -&gt; +35% (L3) -&gt; +42% (L4) -&gt; +50% (L5 Max).
-ATK: -11% -&gt; -14% -&gt; -18% -&gt; -21% -&gt; -25%. TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16.</t>
+          <t>DEF: +20% -&gt; +27% -&gt; +35% -&gt; +42% -&gt; +50% (L1-L5 Max)
+ATK: -11% -&gt; -25%    |    TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1452,8 +1452,8 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Turns: 4 (L1) -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L5 Max). TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24.
-Guard chance: 30%~60% on hit. Requires 1H weapon &amp; shield.</t>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-L5)    |    Guard chance: 30% to 60%
+TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24    |    Requires 1H weapon &amp; shield</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1512,8 +1512,8 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Turns: 3 (L1) -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L5 Max). TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22.
-May break on consecutive blocks. Fast recovery (1.30x speed).</t>
+          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-L5)    |    Recovery Speed: 1.30x
+TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22    |    May break on repeat blocks</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">

</xml_diff>

<commit_message>
fix: clarify accuracy scaling by level and add breathing room spacing
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/skills.xlsx
+++ b/mod_project/data_tables/skills.xlsx
@@ -547,12 +547,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Attract single-target attacks to user. High turn speed recovery.</t>
+          <t>Attract single-target attacks.    |    Fast turn recovery.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-L5)    |    Speed: +50% -&gt; +100%
+          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-5)    |    Speed: +50% -&gt; +100%
 TP Cost: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5</t>
         </is>
       </c>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ATK: +8% -&gt; +10% -&gt; +12% -&gt; +14% -&gt; +18% (L1-L5 Max)
+          <t>ATK: +8% -&gt; +10% -&gt; +12% -&gt; +14% -&gt; +18% (L1-5 Max)
 Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8    |    TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 13</t>
         </is>
       </c>
@@ -711,13 +711,13 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Short-range strike. Boosted accuracy (+20% to +38%). Delay: 0.80x.</t>
+          <t>Short-range strike.    |    Hit Rate: +20% (Lv1) -&gt; +38% (Max)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>ATK: 125% (L1) -&gt; 133 -&gt; 141 -&gt; 150 -&gt; 158 -&gt; 166 -&gt; 175 -&gt; 183 -&gt; 191 -&gt; 200% (L10)
-TP Cost: 5 (L1) -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28 (Max)</t>
+          <t>ATK (L1-10): 125% -&gt; 133 -&gt; 141 -&gt; 150 -&gt; 158 -&gt; 166 -&gt; 175 -&gt; 183 -&gt; 191 -&gt; 200%
+TP Cost: 5 -&gt; 8 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 22 -&gt; 24 -&gt; 26 -&gt; 28  (Lv1 to Max)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>DEF: +20% -&gt; +27% -&gt; +35% -&gt; +42% -&gt; +50% (L1-L5 Max)
+          <t>DEF: +20% -&gt; +27% -&gt; +35% -&gt; +42% -&gt; +50% (L1-5 Max)
 ATK: -11% -&gt; -25%    |    TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix: explicitly specify step (+X/Lv) whenever a range is shown
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/skills.xlsx
+++ b/mod_project/data_tables/skills.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-5)    |    Speed: +50% -&gt; +100%
+          <t>Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 (L1-5)    |    Speed: +50% -&gt; +100% (+12.5%/Lv)
 TP Cost: 1 -&gt; 2 -&gt; 3 -&gt; 4 -&gt; 5</t>
         </is>
       </c>
@@ -711,7 +711,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Short-range strike.    |    Hit Rate: +20% (Lv1) -&gt; +38% (Max)</t>
+          <t>Short-range strike.    |    Hit Rate: +20% -&gt; +38% (+2%/Lv)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -865,7 +865,7 @@
       <c r="J8" t="inlineStr">
         <is>
           <t>DEF: +20% -&gt; +27% -&gt; +35% -&gt; +42% -&gt; +50% (L1-5 Max)
-ATK: -11% -&gt; -25%    |    TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+ATK: -11% -&gt; -25% (-3.5%/Lv)    |    TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-L5)    |    Guard chance: 30% to 60%
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5)    |    Guard: 30% -&gt; 60% (+7.5%/Lv)
 TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 20 -&gt; 24    |    Requires 1H weapon &amp; shield</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: populate complete catalog for Magic User
populate complete catalog for Magic User, Sorceress, and remaining class
skills
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/skills.xlsx
+++ b/mod_project/data_tables/skills.xlsx
@@ -1025,9 +1025,20 @@
 Paralysis rate UP TP Cost UP</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Katana skill. Deal bash damage to one enemy. May paralyze.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 180% (+15%/Lv) | Paralysis: 25% -&gt; 50% (+6.25%/Lv)
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -1069,9 +1080,20 @@
 Duration UP TP Cost UP Enemy critical rate UP</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Greatly boost own critical rate, but increase vulnerability to crits.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Crit Rate: +25% -&gt; +55% (+7.5%/Lv) | Enemy Crit: +15% -&gt; +25%
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2133,9 +2155,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Sword and lance skill. Pierces through to the back row.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>ATK: 135% -&gt; 195% (+15%/Lv) | Hits front and back target
+TP Cost: 12 -&gt; 14 -&gt; 16 -&gt; 18 -&gt; 20</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2535,9 +2568,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Cure status ailments for a single ally.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Cures: Poison (L1) -&gt; Paralyze -&gt; Silence -&gt; Freeze -&gt; Sleep
+TP Cost: 3 -&gt; 5 -&gt; 7 -&gt; 9 -&gt; 11 (L1-5)</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2699,9 +2743,20 @@
 Duration UP TP Cost UP</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Increase own physical evasion and magic evasion.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Physical &amp; Magic EVA: +12% -&gt; +28% (+4%/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3283,9 +3338,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Bow skill. Deal stab damage to one enemy. May slow.</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>ATK: 115% -&gt; 175% (+15%/Lv) | Slow: 25% -&gt; 50% (+6.25%/Lv)
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3551,9 +3617,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Deal bash damage to one enemy. May stun.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>ATK: 130% -&gt; 190% (+15%/Lv) | Stun: 30% -&gt; 60% (+7.5%/Lv)
+TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3594,9 +3671,20 @@
           <t>LvUp: Identification success rate UP TP Cost DOWN</t>
         </is>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Identify unknown dungeon loot items.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Success Rate: 70% -&gt; 98% (+7%/Lv) | Levels: L1-5
+TP Cost: 5 -&gt; 4 -&gt; 3 -&gt; 2 -&gt; 1 (Max)</t>
+        </is>
+      </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3682,9 +3770,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Mace skill. Heavy bash strike with boosted accuracy.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ATK: 140% -&gt; 200% (+15%/Lv) | Accuracy: +25% -&gt; +45% (+5%/Lv)
+TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3726,9 +3825,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Mace skill. Strike target and reduce enemy physical DEF by 10%.</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>ATK: 125% -&gt; 185% (+15%/Lv) | Inflicts -10% DEF debuff
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 | Fast turn recovery (0.85x delay)</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3770,9 +3880,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Sword skill. Deal slash damage to all enemies on screen.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 160% (+10%/Lv, L1-5) | Hits all foes
+TP Cost: 36 -&gt; 46 -&gt; 57 -&gt; 68 -&gt; 79 | Action delay: 0.80x -&gt; 0.98x</t>
+        </is>
+      </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3858,9 +3979,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Transform into Magical Princess, raising all stats.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>All Stats: +15% -&gt; +35% (+5%/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32</t>
+        </is>
+      </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3902,9 +4034,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Short-range strike dealing heavy lightning damage to one enemy.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>ATK: 136% -&gt; 216% (+20%/Lv, L1-5) | Lightning element
+TP Cost: 13 -&gt; 20 -&gt; 28 -&gt; 36 -&gt; 45</t>
+        </is>
+      </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4307,9 +4450,20 @@
           <t>LvUp: TP recovery UP</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Focus divine power to restore own TP.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>TP Restore: 16% -&gt; 25% Max TP (+2.25%/Lv) | Levels: L1-5
+TP Cost: 0 | Action delay: 1.00x</t>
+        </is>
+      </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4350,9 +4504,20 @@
           <t>LvUp: ATK decrease UP</t>
         </is>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Dance skill. Lower all enemies' physical ATK while dance lasts.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Enemy ATK: -12% -&gt; -24% (-3%/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4393,9 +4558,20 @@
           <t>LvUp: DEF decrease UP</t>
         </is>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Dance skill. Lower all enemies' physical DEF while dance lasts.</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Enemy DEF: -12% -&gt; -24% (-3%/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4653,9 +4829,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Whip skill. Deal bash damage to an enemy row from mid-range.</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 180% (+15%/Lv) | Row bash attack
+TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 (L1-5)</t>
+        </is>
+      </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4943,9 +5130,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Attack one enemy. May instakill.</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>ATK: 140% -&gt; 200% (+15%/Lv) | Instakill Chance: 15% -&gt; 35% (+5%/Lv)
+TP Cost: 16 -&gt; 19 -&gt; 22 -&gt; 25 -&gt; 28 (L1-5)</t>
+        </is>
+      </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5031,9 +5229,20 @@
 Time until next turn DOWN TP Cost UP DEF decrease UP</t>
         </is>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Greatly boost own physical ATK at the cost of reducing DEF to 0.</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>ATK: +40% -&gt; +80% (+10%/Lv) | User DEF reduced to 0
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24</t>
+        </is>
+      </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5201,9 +5410,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Fan skill. Deal bash damage to one enemy and delay target turn.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>ATK: 120% -&gt; 180% (+15%/Lv) | Action Delay: -20% -&gt; -40%
+TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5371,9 +5591,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Convert current DEF to bonus ATK (user DEF becomes 0).</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>ATK Bonus: 100% -&gt; 150% of converted DEF value (+12.5%/Lv)
+Turns: 3 -&gt; 4 -&gt; 5 -&gt; 6 -&gt; 7 | TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26</t>
+        </is>
+      </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5497,9 +5728,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Summon puppet Spartan to attack enemies with short-range bash strikes.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Puppet Power: 100% -&gt; 160% (+15%/Lv) | Duration: 4 -&gt; 6 turns
+TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 (L1-5)</t>
+        </is>
+      </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5585,9 +5827,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Summon puppet Catalina to heal party members' HP.</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Heal Potency: 20% -&gt; 40% Max HP (+5%/Lv) | Duration: 4 -&gt; 6 turns
+TP Cost: 14 -&gt; 17 -&gt; 20 -&gt; 23 -&gt; 26 (L1-5)</t>
+        </is>
+      </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5673,9 +5926,20 @@
 petrify &gt; slow &gt; all debuffs TP Cost UP</t>
         </is>
       </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Summon puppet Perdurabo to cure allies' status ailments.</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Cures status ailments for 2 allies per turn | Duration: 4 -&gt; 6 turns
+TP Cost: 12 -&gt; 15 -&gt; 18 -&gt; 21 -&gt; 24 (L1-5)</t>
+        </is>
+      </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5717,9 +5981,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Summon puppet Musiy to cast immediate single-target attack spells.</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Spell Pwr: 120 -&gt; 240 (+30/Lv) | Duration: 4 -&gt; 6 turns
+TP Cost: 16 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 (L1-5)</t>
+        </is>
+      </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7669,9 +7944,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Deal fire damage to an enemy row.</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 90 -&gt; 125 -&gt; 160 -&gt; 200 -&gt; 250 -&gt; 300 -&gt; 360 -&gt; 420 -&gt; 480 -&gt; 530
+TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7713,9 +7999,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Deal fire damage to all enemies.</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 80 -&gt; 110 -&gt; 140 -&gt; 180 -&gt; 230 -&gt; 280 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 510
+TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7757,9 +8054,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Unleash devastating master fire magic on one enemy.</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 620 -&gt; 680 -&gt; 750 -&gt; 830 -&gt; 920 -&gt; 1010 -&gt; 1100 -&gt; 1200 -&gt; 1250 -&gt; 1300
+TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7801,9 +8109,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Deal water damage to one enemy.</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 70 -&gt; 105 -&gt; 140 -&gt; 175 -&gt; 220 -&gt; 270 -&gt; 320 -&gt; 380 -&gt; 450 -&gt; 520
+TP Cost: 5 -&gt; 7 -&gt; 9 -&gt; 11 -&gt; 14 -&gt; 17 -&gt; 20 -&gt; 24 -&gt; 28 -&gt; 32 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7845,9 +8164,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Deal water damage to an enemy row.</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 90 -&gt; 125 -&gt; 160 -&gt; 200 -&gt; 250 -&gt; 300 -&gt; 360 -&gt; 420 -&gt; 480 -&gt; 530
+TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7889,9 +8219,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Deal water damage to all enemies.</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 80 -&gt; 110 -&gt; 140 -&gt; 180 -&gt; 230 -&gt; 280 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 510
+TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7933,9 +8274,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Unleash devastating master water magic on one enemy.</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 620 -&gt; 680 -&gt; 750 -&gt; 830 -&gt; 920 -&gt; 1010 -&gt; 1100 -&gt; 1200 -&gt; 1250 -&gt; 1300
+TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8037,9 +8389,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Deal lightning damage to an enemy row.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 90 -&gt; 125 -&gt; 160 -&gt; 200 -&gt; 250 -&gt; 300 -&gt; 360 -&gt; 420 -&gt; 480 -&gt; 530
+TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8081,9 +8444,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Deal lightning damage to all enemies.</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 80 -&gt; 110 -&gt; 140 -&gt; 180 -&gt; 230 -&gt; 280 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 510
+TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8125,9 +8499,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Unleash devastating master lightning magic on one enemy.</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 620 -&gt; 680 -&gt; 750 -&gt; 830 -&gt; 920 -&gt; 1010 -&gt; 1100 -&gt; 1200 -&gt; 1250 -&gt; 1300
+TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8229,9 +8614,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Deal wind damage to an enemy row.</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 90 -&gt; 125 -&gt; 160 -&gt; 200 -&gt; 250 -&gt; 300 -&gt; 360 -&gt; 420 -&gt; 480 -&gt; 530
+TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8273,9 +8669,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Deal wind damage to all enemies.</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 80 -&gt; 110 -&gt; 140 -&gt; 180 -&gt; 230 -&gt; 280 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 510
+TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8317,9 +8724,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Unleash devastating master wind magic on one enemy.</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 620 -&gt; 680 -&gt; 750 -&gt; 830 -&gt; 920 -&gt; 1010 -&gt; 1100 -&gt; 1200 -&gt; 1250 -&gt; 1300
+TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8421,9 +8839,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Deal earth damage to an enemy row.</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 90 -&gt; 125 -&gt; 160 -&gt; 200 -&gt; 250 -&gt; 300 -&gt; 360 -&gt; 420 -&gt; 480 -&gt; 530
+TP Cost: 15 -&gt; 19 -&gt; 23 -&gt; 27 -&gt; 32 -&gt; 37 -&gt; 43 -&gt; 49 -&gt; 55 -&gt; 60 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8465,9 +8894,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Deal earth damage to all enemies.</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 80 -&gt; 110 -&gt; 140 -&gt; 180 -&gt; 230 -&gt; 280 -&gt; 340 -&gt; 400 -&gt; 460 -&gt; 510
+TP Cost: 25 -&gt; 30 -&gt; 35 -&gt; 41 -&gt; 48 -&gt; 55 -&gt; 63 -&gt; 71 -&gt; 79 -&gt; 88 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8509,9 +8949,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Unleash devastating master earth magic on one enemy.</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Pwr (L1-10): 620 -&gt; 680 -&gt; 750 -&gt; 830 -&gt; 920 -&gt; 1010 -&gt; 1100 -&gt; 1200 -&gt; 1250 -&gt; 1300
+TP Cost: 40 -&gt; 44 -&gt; 48 -&gt; 53 -&gt; 58 -&gt; 64 -&gt; 70 -&gt; 76 -&gt; 80 -&gt; 84 (Lv1 to Max)</t>
+        </is>
+      </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8553,9 +9004,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Neutral magic strike to one enemy. Absorb damage dealt as HP.</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Pwr: 60 -&gt; 120 -&gt; 180 -&gt; 260 -&gt; 350 (L1-5) | Bypasses elemental resists
+TP Cost: 9 -&gt; 11 -&gt; 13 -&gt; 15 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8597,9 +9059,20 @@
 TP Cost UP Chant time UP</t>
         </is>
       </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Neutral magic strike to one enemy. Absorb damage dealt as TP.</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Pwr: 22 -&gt; 35 -&gt; 50 -&gt; 65 -&gt; 82 (L1-5) | Restores TP equal to damage dealt
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 15</t>
+        </is>
+      </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8641,9 +9114,20 @@
 Duration UP TP Cost UP</t>
         </is>
       </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Boost own magic attack power at the cost of consuming HP.</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Magic ATK: +20% -&gt; +40% (+5%/Lv) | HP Cost: 10% Max HP
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8685,9 +9169,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Transfer a portion of user HP to restore an ally's HP.</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Heal: 30% -&gt; 60% (+7.5%/Lv) of target Max HP | Consumes 20% user HP
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16 (L1-5)</t>
+        </is>
+      </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8729,9 +9224,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Deal magic damage to one enemy. May stun.</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Stun Chance: 30% -&gt; 60% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8773,9 +9279,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Poison all enemies (5% Max HP damage per enemy turn, cap 250).</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Accuracy: +15% -&gt; +35% (+5%/Lv) | Chant: 1.20x -&gt; 1.40x
+TP Cost: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5)</t>
+        </is>
+      </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8817,9 +9334,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Deal water magic damage to one enemy. May freeze.</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Freeze Chance: 30% -&gt; 60% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8861,9 +9389,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Deal lightning magic damage to one enemy. May paralyze.</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Paralysis Chance: 30% -&gt; 60% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8905,9 +9444,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Put an enemy to sleep with magic.</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Sleep Chance: 40% -&gt; 70% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8949,9 +9499,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Silence an enemy to prevent spell casting.</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Silence Chance: 40% -&gt; 70% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8993,9 +9554,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Turn one enemy to stone with earth magic.</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Petrify Chance: 20% -&gt; 40% (+5%/Lv) | Levels: L1-5
+TP Cost: 10 -&gt; 13 -&gt; 16 -&gt; 19 -&gt; 22</t>
+        </is>
+      </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9037,9 +9609,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Attempt to instantly slay one living enemy.</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Instakill Chance: 15% -&gt; 35% (+5%/Lv) | Levels: L1-5
+TP Cost: 15 -&gt; 18 -&gt; 21 -&gt; 24 -&gt; 28</t>
+        </is>
+      </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9081,9 +9664,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Inflict Slow on an enemy row, cutting action speed by -50%.</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Slow Chance: 35% -&gt; 65% (+7.5%/Lv) | Inflicts -50% Speed
+TP Cost: 15 -&gt; 17 -&gt; 19 -&gt; 21 -&gt; 23 (L1-5)</t>
+        </is>
+      </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9125,9 +9719,20 @@
 TP Cost UP</t>
         </is>
       </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Terrify an enemy with dark magic to inflict Stun.</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Stun Chance: 30% -&gt; 60% (+7.5%/Lv) | Levels: L1-5
+TP Cost: 8 -&gt; 10 -&gt; 12 -&gt; 14 -&gt; 16</t>
+        </is>
+      </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9257,9 +9862,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Imbue an ally's weapon with Fire element.</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5) | Adds Fire damage to weapon strikes
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9301,9 +9917,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Imbue an ally's weapon with Water element.</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5) | Adds Water damage to weapon strikes
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9345,9 +9972,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Imbue an ally's weapon with Lightning element.</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5) | Adds Lightning damage to weapon strikes
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9389,9 +10027,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Imbue an ally's weapon with Wind element.</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5) | Adds Wind damage to weapon strikes
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9433,9 +10082,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Imbue an ally's weapon with Earth element.</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 (L1-5) | Adds Earth damage to weapon strikes
+TP Cost: 6 -&gt; 8 -&gt; 10 -&gt; 12 -&gt; 14</t>
+        </is>
+      </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9477,9 +10137,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Raise one row of allies' resistance to stab damage.</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>Stab Resistance: +15 -&gt; +35 (+5/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9521,9 +10192,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Raise one row of allies' resistance to slash damage.</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>Slash Resistance: +15 -&gt; +35 (+5/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9565,9 +10247,20 @@
 Time until next turn DOWN TP Cost UP</t>
         </is>
       </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Raise one row of allies' resistance to bash damage.</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>Bash Resistance: +15 -&gt; +35 (+5/Lv) | Levels: L1-5
+Turns: 4 -&gt; 5 -&gt; 6 -&gt; 7 -&gt; 8 | TP Cost: 10 -&gt; 12 -&gt; 14 -&gt; 16 -&gt; 18</t>
+        </is>
+      </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14330,9 +15023,20 @@
           <t>LvUp: Activation rate UP</t>
         </is>
       </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Occasionally nullify physical damage.</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Nullify Rate: 8% -&gt; 20% (+3%/Lv) | Levels: L1-5
+Completely negates incoming physical attacks when triggered</t>
+        </is>
+      </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14373,9 +15077,20 @@
           <t>LvUp: Can cure poison &gt; paralysis &gt; silence &gt; freeze &gt; sleep &gt; slow</t>
         </is>
       </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Automatically cure own status ailments at start of turn.</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>Cures: Poison (L1) -&gt; Paralyze -&gt; Silence -&gt; Freeze -&gt; Sleep -&gt; Slow
+Triggers automatically at start of user's combat turn</t>
+        </is>
+      </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14416,9 +15131,20 @@
           <t>LvUp: ATK/DEX increase UP</t>
         </is>
       </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Boost physical ATK and DEX when HP drops below 50%.</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>ATK &amp; DEX: +20% -&gt; +40% (+5%/Lv) when HP &lt; 50% | Levels: L1-5
+Immediate combat stat trigger</t>
+        </is>
+      </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14636,9 +15362,20 @@
           <t>LvUp: Accuracy UP</t>
         </is>
       </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Heighten magic accuracy for all cast spells.</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>Magic Accuracy: +15% -&gt; +35% (+5%/Lv) | Levels: L1-5
+Significantly reduces spell evasion by high RES targets</t>
+        </is>
+      </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14679,9 +15416,20 @@
           <t>LvUp: Enemy preemptive attack rate DOWN</t>
         </is>
       </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Reduce enemy preemptive strike rate in dungeons.</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>Preemptive Reduction: -20% -&gt; -60% (-10%/Lv) | Levels: L1-5
+Protects party from surprise enemy encounters</t>
+        </is>
+      </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14722,9 +15470,20 @@
           <t>LvUp: Preemptive attack rate UP</t>
         </is>
       </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Increase party's preemptive strike rate against foes.</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>Party Preemptive Rate: +10% -&gt; +30% (+5%/Lv) | Levels: L1-5
+Grants free initial turn before enemies act</t>
+        </is>
+      </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14765,9 +15524,20 @@
           <t>LvUp: Battle escape rate UP</t>
         </is>
       </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Increase success rate when attempting to flee from battle.</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>Escape Success: +20% -&gt; +50% (+7.5%/Lv) | Levels: L1-5
+Does not apply to scripted boss battles</t>
+        </is>
+      </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14926,9 +15696,20 @@
           <t>LvUp: Found item quality UP</t>
         </is>
       </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Occasionally discover items while exploring dungeons.</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>Item Find Rate: +10% -&gt; +30% (+5%/Lv) | Levels: L1-5
+Finds consumables and crafting materials while walking</t>
+        </is>
+      </c>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -14969,9 +15750,20 @@
           <t>LvUp: Post-battle HP &amp; TP recovery UP</t>
         </is>
       </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Restore party HP and TP slightly after winning a battle.</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery: 5% -&gt; 15% HP &amp; TP (+2.5%/Lv) | Levels: L1-5
+Restores whole party after combat conclusion</t>
+        </is>
+      </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15012,9 +15804,20 @@
           <t>LvUp: Item keep rate UP</t>
         </is>
       </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Occasionally retain disposable items after using them in combat.</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>Item Retain Chance: 15% -&gt; 35% (+5%/Lv) | Levels: L1-5
+Item is not consumed from inventory when triggered</t>
+        </is>
+      </c>
       <c r="K294" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15114,9 +15917,20 @@
           <t>LvUp: Speed UP</t>
         </is>
       </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Become capable of performing two songs simultaneously.</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Singing Speed: +10% -&gt; +30% (+5%/Lv) | Levels: L1-5
+Allows maintaining 2 active Bard songs at once</t>
+        </is>
+      </c>
       <c r="K296" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15157,9 +15971,20 @@
           <t>LvUp: Speed UP</t>
         </is>
       </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Become capable of performing two dances simultaneously.</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Dancing Speed: +10% -&gt; +30% (+5%/Lv) | Levels: L1-5
+Allows maintaining 2 active Dancer dances at once</t>
+        </is>
+      </c>
       <c r="K297" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15200,9 +16025,20 @@
           <t>LvUp: Speed UP</t>
         </is>
       </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Become capable of controlling two summoned dolls at once.</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Doll Control Speed: +10% -&gt; +30% (+5%/Lv) | Levels: L1-5
+Maintains 2 active summoned dolls simultaneously</t>
+        </is>
+      </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15243,9 +16079,20 @@
           <t>LvUp: Sealbook ability increase UP</t>
         </is>
       </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Increase doll power with strength of equipped Sealbook.</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>Doll Power Bonus: +10% -&gt; +30% (+5%/Lv) based on Sealbook level
+Levels: L1-5</t>
+        </is>
+      </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15463,9 +16310,20 @@
           <t>LvUp: Doll skill bonus UP</t>
         </is>
       </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Increased potency and effectiveness for all doll skills.</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Doll Stat Bonus: +3% -&gt; +15% (+3%/Lv) | Levels: L1-5
+Increases damage, healing, and durability of summoned dolls</t>
+        </is>
+      </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15506,9 +16364,20 @@
           <t>LvUp: Double attack rate UP</t>
         </is>
       </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Occasionally attack twice when performing normal attacks.</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Double Attack Rate: 8% -&gt; 20% (+3%/Lv) | Levels: L1-5
+Normal attack trigger</t>
+        </is>
+      </c>
       <c r="K304" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15549,9 +16418,20 @@
           <t>LvUp: Song chant time DOWN</t>
         </is>
       </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Reduce chant time required to start songs.</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Song Chant Reduction: -10% -&gt; -30% (-5%/Lv) | Levels: L1-5
+Accelerates Bard song activation</t>
+        </is>
+      </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15592,9 +16472,20 @@
           <t>LvUp: Negotiation rate UP</t>
         </is>
       </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Reduce purchase and identification prices at shops.</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Shop Discount: -5% -&gt; -25% (-5%/Lv) | Levels: L1-5
+Lowers gold cost for item purchases and item identification</t>
+        </is>
+      </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15635,9 +16526,20 @@
           <t>LvUp: Occurrence rate UP</t>
         </is>
       </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Mesmerize enemies with dance steps, causing them to lose turns.</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Mesmerize Rate: 5% -&gt; 15% (+2.5%/Lv) | Levels: L1-5
+Enemy skips turn when mesmerized</t>
+        </is>
+      </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15673,9 +16575,20 @@
           <t>Nullify first hit of battle against user (does not work for status ailments).</t>
         </is>
       </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Nullify first hit of battle against user.</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>100% nullification of the very first physical attack received
+Fixed passive (Level 1)</t>
+        </is>
+      </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15711,9 +16624,20 @@
           <t>Heighten the probability of beneficial results for random effect skills.</t>
         </is>
       </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Heighten probability of beneficial results for random skills.</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Drastically increases odds of favorable outcomes on Gamble skills
+Fixed passive (Level 1)</t>
+        </is>
+      </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15879,9 +16803,20 @@
           <t>Increase doll summon duration by 1 turn.</t>
         </is>
       </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Increase doll summon duration on battlefield.</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Doll Summon Duration: +1 turn (Summons persist longer in battle)
+Fixed passive (Level 1)</t>
+        </is>
+      </c>
       <c r="K313" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -15923,7 +16858,6 @@
 Effect: +1% damage per Pep point (up to +100% damage at Max Pep).</t>
         </is>
       </c>
-      <c r="J314" t="inlineStr"/>
       <c r="K314" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -15973,7 +16907,6 @@
 Inflicts Poison, Paralyze, Silence, or cancels enemy buffs.</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr"/>
       <c r="K315" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16023,7 +16956,6 @@
 Inflicts Slow and -30% Speed on attacker.</t>
         </is>
       </c>
-      <c r="J316" t="inlineStr"/>
       <c r="K316" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16073,7 +17005,6 @@
 Grants +25% extra damage to all weapon-based techniques.</t>
         </is>
       </c>
-      <c r="J317" t="inlineStr"/>
       <c r="K317" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16123,7 +17054,6 @@
 Guarantees 100% hit rate and completely ignores target DEF.</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr"/>
       <c r="K318" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16173,7 +17103,6 @@
 Chance to completely negate all incoming damage.</t>
         </is>
       </c>
-      <c r="J319" t="inlineStr"/>
       <c r="K319" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16223,7 +17152,6 @@
 Instantly eliminates enemy summon entities, puppets, and familiars.</t>
         </is>
       </c>
-      <c r="J320" t="inlineStr"/>
       <c r="K320" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16273,7 +17201,6 @@
 Uses a free recovery item from personal stock without turn cost.</t>
         </is>
       </c>
-      <c r="J321" t="inlineStr"/>
       <c r="K321" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16323,7 +17250,6 @@
 Decreases action recovery delay by 20% after using skills or magic.</t>
         </is>
       </c>
-      <c r="J322" t="inlineStr"/>
       <c r="K322" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16373,7 +17299,6 @@
 Increases potency and effectiveness of all Maid skills by +15%.</t>
         </is>
       </c>
-      <c r="J323" t="inlineStr"/>
       <c r="K323" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16423,7 +17348,6 @@
 Grants an immediate second action in the same turn.</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
       <c r="K324" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16473,7 +17397,6 @@
 Resurrects with 50% Max HP 3 turns after falling in combat.</t>
         </is>
       </c>
-      <c r="J325" t="inlineStr"/>
       <c r="K325" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16523,7 +17446,6 @@
 Reduces incoming damage from Demons, Undead, and Apparitions by 20%.</t>
         </is>
       </c>
-      <c r="J326" t="inlineStr"/>
       <c r="K326" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16573,7 +17495,6 @@
 Inflicts -20% ATK and -20% INT on all enemies.</t>
         </is>
       </c>
-      <c r="J327" t="inlineStr"/>
       <c r="K327" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16623,7 +17544,6 @@
 Offensive and support spells activate immediately with 0 chant time.</t>
         </is>
       </c>
-      <c r="J328" t="inlineStr"/>
       <c r="K328" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16673,7 +17593,6 @@
 Reflects 30% of received damage back to attacker as neutral damage.</t>
         </is>
       </c>
-      <c r="J329" t="inlineStr"/>
       <c r="K329" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16723,7 +17642,6 @@
 Normal attacks trigger an extra strike dealing 75% damage.</t>
         </is>
       </c>
-      <c r="J330" t="inlineStr"/>
       <c r="K330" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -16773,7 +17691,6 @@
 Increases all class stat bonuses and weapon masteries by +10%.</t>
         </is>
       </c>
-      <c r="J331" t="inlineStr"/>
       <c r="K331" t="inlineStr">
         <is>
           <t>Approved</t>

</xml_diff>

<commit_message>
feat: implement equipment transparency
implement equipment transparency (551 items) and Crown EX unique skills
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/skills.xlsx
+++ b/mod_project/data_tables/skills.xlsx
@@ -16871,7 +16871,8 @@
       <c r="I314" t="inlineStr">
         <is>
           <t>Heroine: Luco | Damage scales with Pep.
-Effect: +1% damage per Pep point (up to +100% damage at Max Pep).</t>
+Effect: +1% damage per Pep point (up to +100% damage at Max Pep).
+[Crown EX]: Scales up to +150% damage bonus at Max Pep.</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
@@ -16920,7 +16921,8 @@
       <c r="I315" t="inlineStr">
         <is>
           <t>Heroine: Mefmera | 15% trigger chance on enemy action.
-Inflicts Poison, Paralyze, Silence, or cancels enemy buffs.</t>
+Inflicts Poison, Paralyze, Silence, or cancels enemy buffs.
+[Crown EX]: Trigger chance increases to 25% on any enemy action.</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -16969,7 +16971,8 @@
       <c r="I316" t="inlineStr">
         <is>
           <t>Heroine: Souffle | 25% counter chance on physical contact.
-Inflicts Slow and -30% Speed on attacker.</t>
+Inflicts Slow and -30% Speed on attacker.
+[Crown EX]: Counter chance increases to 40% on physical contact.</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -17018,7 +17021,8 @@
       <c r="I317" t="inlineStr">
         <is>
           <t>Heroine: Grishna | Weapon Scaling Bonus.
-Grants +25% extra damage to all weapon-based techniques.</t>
+Grants +25% extra damage to all weapon-based techniques.
+[Crown EX]: Weapon technique damage bonus increases to +40%.</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -17067,7 +17071,8 @@
       <c r="I318" t="inlineStr">
         <is>
           <t>Heroine: Yae | 20% activation rate on physical attacks.
-Guarantees 100% hit rate and completely ignores target DEF.</t>
+Guarantees 100% hit rate and completely ignores target DEF.
+[Crown EX]: Activation rate increases to 30% (ignores target DEF).</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -17116,7 +17121,8 @@
       <c r="I319" t="inlineStr">
         <is>
           <t>Heroine: Lize | 10% nullification rate.
-Chance to completely negate all incoming damage.</t>
+Chance to completely negate all incoming damage.
+[Crown EX]: Total damage nullification rate increases to 15%.</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -17165,7 +17171,8 @@
       <c r="I320" t="inlineStr">
         <is>
           <t>Heroine: Lilian | 25% banish rate before acting.
-Instantly eliminates enemy summon entities, puppets, and familiars.</t>
+Instantly eliminates enemy summon entities, puppets, and familiars.
+[Crown EX]: Enemy summon and minion banish rate increases to 40%.</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
@@ -17214,7 +17221,8 @@
       <c r="I321" t="inlineStr">
         <is>
           <t>Heroine: Monica | 20% trigger rate at start of turn.
-Uses a free recovery item from personal stock without turn cost.</t>
+Uses a free recovery item from personal stock without turn cost.
+[Crown EX]: Free item trigger rate increases to 30% without turn cost.</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -17263,7 +17271,8 @@
       <c r="I322" t="inlineStr">
         <is>
           <t>Heroine: Alisia | Action Recovery Acceleration.
-Decreases action recovery delay by 20% after using skills or magic.</t>
+Decreases action recovery delay by 20% after using skills or magic.
+[Crown EX]: Action recovery delay reduction increases to 30%.</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
@@ -17312,7 +17321,8 @@
       <c r="I323" t="inlineStr">
         <is>
           <t>Heroine: Conette | Maid Mastery Booster.
-Increases potency and effectiveness of all Maid skills by +15%.</t>
+Increases potency and effectiveness of all Maid skills by +15%.
+[Crown EX]: Maid skill effectiveness bonus increases to +25%.</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
@@ -17361,7 +17371,8 @@
       <c r="I324" t="inlineStr">
         <is>
           <t>Heroine: Yuni | 15% double action chance.
-Grants an immediate second action in the same turn.</t>
+Grants an immediate second action in the same turn.
+[Crown EX]: Immediate second action trigger rate increases to 25%.</t>
         </is>
       </c>
       <c r="K324" t="inlineStr">
@@ -17410,7 +17421,8 @@
       <c r="I325" t="inlineStr">
         <is>
           <t>Heroine: Gina | Auto-Resurrection.
-Resurrects with 50% Max HP 3 turns after falling in combat.</t>
+Resurrects with 50% Max HP 3 turns after falling in combat.
+[Crown EX]: Resurrects with 100% Max HP after 2 turns.</t>
         </is>
       </c>
       <c r="K325" t="inlineStr">
@@ -17459,7 +17471,8 @@
       <c r="I326" t="inlineStr">
         <is>
           <t>Heroine: Ist | Row Protection Barrier.
-Reduces incoming damage from Demons, Undead, and Apparitions by 20%.</t>
+Reduces incoming damage from Demons, Undead, and Apparitions by 20%.
+[Crown EX]: Damage reduction from Demons/Undead/Apparitions to 30%.</t>
         </is>
       </c>
       <c r="K326" t="inlineStr">
@@ -17508,7 +17521,8 @@
       <c r="I327" t="inlineStr">
         <is>
           <t>Heroine: Fiora | 15% trigger rate at start of turn.
-Inflicts -20% ATK and -20% INT on all enemies.</t>
+Inflicts -20% ATK and -20% INT on all enemies.
+[Crown EX]: Turn-start debuff trigger rate increases to 25%.</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
@@ -17557,7 +17571,8 @@
       <c r="I328" t="inlineStr">
         <is>
           <t>Heroine: Eltricia | 15% instant cast chance.
-Offensive and support spells activate immediately with 0 chant time.</t>
+Offensive and support spells activate immediately with 0 chant time.
+[Crown EX]: Instant cast (0 chant delay) rate increases to 25%.</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
@@ -17606,7 +17621,8 @@
       <c r="I329" t="inlineStr">
         <is>
           <t>Heroine: Melvy | 20% damage reflect rate.
-Reflects 30% of received damage back to attacker as neutral damage.</t>
+Reflects 30% of received damage back to attacker as neutral damage.
+[Crown EX]: Damage reflect rate increases to 30% with 45% reflected.</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -17655,7 +17671,8 @@
       <c r="I330" t="inlineStr">
         <is>
           <t>Heroine: Tsurara | Shadow Clone Follow-up.
-Normal attacks trigger an extra strike dealing 75% damage.</t>
+Normal attacks trigger an extra strike dealing 75% damage.
+[Crown EX]: Shadow strike follow-up deals 100% full attack damage.</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
@@ -17704,7 +17721,8 @@
       <c r="I331" t="inlineStr">
         <is>
           <t>Heroine: Siena | Class Mastery Booster.
-Increases all class stat bonuses and weapon masteries by +10%.</t>
+Increases all class stat bonuses and weapon masteries by +10%.
+[Crown EX]: Class and weapon mastery bonuses increase to +15%.</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">

</xml_diff>